<commit_message>
ultima validacion - paper
</commit_message>
<xml_diff>
--- a/Proyecto Interno/review-food-security-paper/00_pipeline/robust/threshold_grid_results.xlsx
+++ b/Proyecto Interno/review-food-security-paper/00_pipeline/robust/threshold_grid_results.xlsx
@@ -438,28 +438,28 @@
         <v>3</v>
       </c>
       <c r="D2">
-        <v>8.187502353415857</v>
+        <v>8.12025866908364</v>
       </c>
       <c r="E2">
         <v>8.008194577779713</v>
       </c>
       <c r="F2">
-        <v>-0.1793077756361434</v>
+        <v>-0.1120640913039264</v>
       </c>
       <c r="G2">
-        <v>8.187502353415857</v>
+        <v>9.721543496423253</v>
       </c>
       <c r="H2">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I2">
-        <v>-0.1793077756361434</v>
+        <v>-0.1463257243140426</v>
       </c>
       <c r="J2">
-        <v>3796</v>
+        <v>2704</v>
       </c>
       <c r="K2">
-        <v>1456</v>
+        <v>1378</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -482,28 +482,28 @@
         <v>3</v>
       </c>
       <c r="D3">
-        <v>8.187502353415857</v>
+        <v>8.12025866908364</v>
       </c>
       <c r="E3">
         <v>8.008194577779713</v>
       </c>
       <c r="F3">
-        <v>-0.1793077756361434</v>
+        <v>-0.1120640913039264</v>
       </c>
       <c r="G3">
-        <v>8.187502353415857</v>
+        <v>9.721543496423253</v>
       </c>
       <c r="H3">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I3">
-        <v>-0.1793077756361434</v>
+        <v>-0.1463257243140426</v>
       </c>
       <c r="J3">
-        <v>3796</v>
+        <v>2704</v>
       </c>
       <c r="K3">
-        <v>1456</v>
+        <v>1378</v>
       </c>
       <c r="L3">
         <v>0</v>
@@ -526,28 +526,28 @@
         <v>3</v>
       </c>
       <c r="D4">
-        <v>8.187502353415857</v>
+        <v>8.12025866908364</v>
       </c>
       <c r="E4">
         <v>8.008194577779713</v>
       </c>
       <c r="F4">
-        <v>-0.1793077756361434</v>
+        <v>-0.1120640913039264</v>
       </c>
       <c r="G4">
-        <v>8.187502353415857</v>
+        <v>9.721543496423253</v>
       </c>
       <c r="H4">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I4">
-        <v>-0.1793077756361434</v>
+        <v>-0.1463257243140426</v>
       </c>
       <c r="J4">
-        <v>3796</v>
+        <v>2704</v>
       </c>
       <c r="K4">
-        <v>1456</v>
+        <v>1378</v>
       </c>
       <c r="L4">
         <v>0</v>
@@ -570,28 +570,28 @@
         <v>4</v>
       </c>
       <c r="D5">
-        <v>8.187502353415857</v>
+        <v>8.12025866908364</v>
       </c>
       <c r="E5">
         <v>8.008194577779713</v>
       </c>
       <c r="F5">
-        <v>-0.1793077756361434</v>
+        <v>-0.1120640913039264</v>
       </c>
       <c r="G5">
-        <v>8.187502353415857</v>
+        <v>9.721543496423253</v>
       </c>
       <c r="H5">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I5">
-        <v>-0.1793077756361434</v>
+        <v>-0.1463257243140426</v>
       </c>
       <c r="J5">
-        <v>3796</v>
+        <v>2704</v>
       </c>
       <c r="K5">
-        <v>1456</v>
+        <v>1378</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -614,28 +614,28 @@
         <v>4</v>
       </c>
       <c r="D6">
-        <v>8.187502353415857</v>
+        <v>8.12025866908364</v>
       </c>
       <c r="E6">
         <v>8.008194577779713</v>
       </c>
       <c r="F6">
-        <v>-0.1793077756361434</v>
+        <v>-0.1120640913039264</v>
       </c>
       <c r="G6">
-        <v>8.187502353415857</v>
+        <v>9.721543496423253</v>
       </c>
       <c r="H6">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I6">
-        <v>-0.1793077756361434</v>
+        <v>-0.1463257243140426</v>
       </c>
       <c r="J6">
-        <v>3796</v>
+        <v>2704</v>
       </c>
       <c r="K6">
-        <v>1456</v>
+        <v>1378</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -658,28 +658,28 @@
         <v>4</v>
       </c>
       <c r="D7">
-        <v>8.187502353415857</v>
+        <v>8.12025866908364</v>
       </c>
       <c r="E7">
         <v>8.008194577779713</v>
       </c>
       <c r="F7">
-        <v>-0.1793077756361434</v>
+        <v>-0.1120640913039264</v>
       </c>
       <c r="G7">
-        <v>8.187502353415857</v>
+        <v>9.721543496423253</v>
       </c>
       <c r="H7">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I7">
-        <v>-0.1793077756361434</v>
+        <v>-0.1463257243140426</v>
       </c>
       <c r="J7">
-        <v>3796</v>
+        <v>2704</v>
       </c>
       <c r="K7">
-        <v>1456</v>
+        <v>1378</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -702,28 +702,28 @@
         <v>5</v>
       </c>
       <c r="D8">
-        <v>8.187502353415857</v>
+        <v>8.12025866908364</v>
       </c>
       <c r="E8">
         <v>8.008194577779713</v>
       </c>
       <c r="F8">
-        <v>-0.1793077756361434</v>
+        <v>-0.1120640913039264</v>
       </c>
       <c r="G8">
-        <v>8.187502353415857</v>
+        <v>9.721543496423253</v>
       </c>
       <c r="H8">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I8">
-        <v>-0.1793077756361434</v>
+        <v>-0.1463257243140426</v>
       </c>
       <c r="J8">
-        <v>3796</v>
+        <v>2704</v>
       </c>
       <c r="K8">
-        <v>1456</v>
+        <v>1378</v>
       </c>
       <c r="L8">
         <v>0</v>
@@ -746,28 +746,28 @@
         <v>5</v>
       </c>
       <c r="D9">
-        <v>8.187502353415857</v>
+        <v>8.12025866908364</v>
       </c>
       <c r="E9">
         <v>8.008194577779713</v>
       </c>
       <c r="F9">
-        <v>-0.1793077756361434</v>
+        <v>-0.1120640913039264</v>
       </c>
       <c r="G9">
-        <v>8.187502353415857</v>
+        <v>9.721543496423253</v>
       </c>
       <c r="H9">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I9">
-        <v>-0.1793077756361434</v>
+        <v>-0.1463257243140426</v>
       </c>
       <c r="J9">
-        <v>3796</v>
+        <v>2704</v>
       </c>
       <c r="K9">
-        <v>1456</v>
+        <v>1378</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -790,28 +790,28 @@
         <v>5</v>
       </c>
       <c r="D10">
-        <v>8.187502353415857</v>
+        <v>8.12025866908364</v>
       </c>
       <c r="E10">
         <v>8.008194577779713</v>
       </c>
       <c r="F10">
-        <v>-0.1793077756361434</v>
+        <v>-0.1120640913039264</v>
       </c>
       <c r="G10">
-        <v>8.187502353415857</v>
+        <v>9.721543496423253</v>
       </c>
       <c r="H10">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I10">
-        <v>-0.1793077756361434</v>
+        <v>-0.1463257243140426</v>
       </c>
       <c r="J10">
-        <v>3796</v>
+        <v>2704</v>
       </c>
       <c r="K10">
-        <v>1456</v>
+        <v>1378</v>
       </c>
       <c r="L10">
         <v>0</v>
@@ -834,28 +834,28 @@
         <v>3</v>
       </c>
       <c r="D11">
-        <v>8.229678115136942</v>
+        <v>8.147932790882336</v>
       </c>
       <c r="E11">
         <v>8.008194577779713</v>
       </c>
       <c r="F11">
-        <v>-0.2214835373572281</v>
+        <v>-0.139738213102623</v>
       </c>
       <c r="G11">
-        <v>8.229678115136942</v>
+        <v>9.757678496224099</v>
       </c>
       <c r="H11">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I11">
-        <v>-0.2214835373572281</v>
+        <v>-0.1824607241148879</v>
       </c>
       <c r="J11">
-        <v>4628</v>
+        <v>3536</v>
       </c>
       <c r="K11">
-        <v>624</v>
+        <v>546</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -878,28 +878,28 @@
         <v>4</v>
       </c>
       <c r="D12">
-        <v>8.229678115136942</v>
+        <v>8.147932790882336</v>
       </c>
       <c r="E12">
         <v>8.008194577779713</v>
       </c>
       <c r="F12">
-        <v>-0.2214835373572281</v>
+        <v>-0.139738213102623</v>
       </c>
       <c r="G12">
-        <v>8.229678115136942</v>
+        <v>9.757678496224099</v>
       </c>
       <c r="H12">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I12">
-        <v>-0.2214835373572281</v>
+        <v>-0.1824607241148879</v>
       </c>
       <c r="J12">
-        <v>4628</v>
+        <v>3536</v>
       </c>
       <c r="K12">
-        <v>624</v>
+        <v>546</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -922,28 +922,28 @@
         <v>5</v>
       </c>
       <c r="D13">
-        <v>8.229678115136942</v>
+        <v>8.147932790882336</v>
       </c>
       <c r="E13">
         <v>8.008194577779713</v>
       </c>
       <c r="F13">
-        <v>-0.2214835373572281</v>
+        <v>-0.139738213102623</v>
       </c>
       <c r="G13">
-        <v>8.229678115136942</v>
+        <v>9.757678496224099</v>
       </c>
       <c r="H13">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I13">
-        <v>-0.2214835373572281</v>
+        <v>-0.1824607241148879</v>
       </c>
       <c r="J13">
-        <v>4628</v>
+        <v>3536</v>
       </c>
       <c r="K13">
-        <v>624</v>
+        <v>546</v>
       </c>
       <c r="L13">
         <v>0</v>
@@ -966,28 +966,28 @@
         <v>3</v>
       </c>
       <c r="D14">
-        <v>8.239827565084084</v>
+        <v>8.158019721703413</v>
       </c>
       <c r="E14">
         <v>8.008194577779713</v>
       </c>
       <c r="F14">
-        <v>-0.231632987304371</v>
+        <v>-0.1498251439236995</v>
       </c>
       <c r="G14">
-        <v>8.239827565084084</v>
+        <v>9.770849329461811</v>
       </c>
       <c r="H14">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I14">
-        <v>-0.231632987304371</v>
+        <v>-0.1956315573526002</v>
       </c>
       <c r="J14">
-        <v>4186</v>
+        <v>3094</v>
       </c>
       <c r="K14">
-        <v>1066</v>
+        <v>988</v>
       </c>
       <c r="L14">
         <v>0</v>
@@ -1010,28 +1010,28 @@
         <v>3</v>
       </c>
       <c r="D15">
-        <v>8.239827565084084</v>
+        <v>8.158019721703413</v>
       </c>
       <c r="E15">
         <v>8.008194577779713</v>
       </c>
       <c r="F15">
-        <v>-0.231632987304371</v>
+        <v>-0.1498251439236995</v>
       </c>
       <c r="G15">
-        <v>8.239827565084084</v>
+        <v>9.770849329461811</v>
       </c>
       <c r="H15">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I15">
-        <v>-0.231632987304371</v>
+        <v>-0.1956315573526002</v>
       </c>
       <c r="J15">
-        <v>4186</v>
+        <v>3094</v>
       </c>
       <c r="K15">
-        <v>1066</v>
+        <v>988</v>
       </c>
       <c r="L15">
         <v>0</v>
@@ -1054,28 +1054,28 @@
         <v>4</v>
       </c>
       <c r="D16">
-        <v>8.239827565084084</v>
+        <v>8.158019721703413</v>
       </c>
       <c r="E16">
         <v>8.008194577779713</v>
       </c>
       <c r="F16">
-        <v>-0.231632987304371</v>
+        <v>-0.1498251439236995</v>
       </c>
       <c r="G16">
-        <v>8.239827565084084</v>
+        <v>9.770849329461811</v>
       </c>
       <c r="H16">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I16">
-        <v>-0.231632987304371</v>
+        <v>-0.1956315573526002</v>
       </c>
       <c r="J16">
-        <v>4186</v>
+        <v>3094</v>
       </c>
       <c r="K16">
-        <v>1066</v>
+        <v>988</v>
       </c>
       <c r="L16">
         <v>0</v>
@@ -1098,28 +1098,28 @@
         <v>4</v>
       </c>
       <c r="D17">
-        <v>8.239827565084084</v>
+        <v>8.158019721703413</v>
       </c>
       <c r="E17">
         <v>8.008194577779713</v>
       </c>
       <c r="F17">
-        <v>-0.231632987304371</v>
+        <v>-0.1498251439236995</v>
       </c>
       <c r="G17">
-        <v>8.239827565084084</v>
+        <v>9.770849329461811</v>
       </c>
       <c r="H17">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I17">
-        <v>-0.231632987304371</v>
+        <v>-0.1956315573526002</v>
       </c>
       <c r="J17">
-        <v>4186</v>
+        <v>3094</v>
       </c>
       <c r="K17">
-        <v>1066</v>
+        <v>988</v>
       </c>
       <c r="L17">
         <v>0</v>
@@ -1142,28 +1142,28 @@
         <v>5</v>
       </c>
       <c r="D18">
-        <v>8.239827565084084</v>
+        <v>8.158019721703413</v>
       </c>
       <c r="E18">
         <v>8.008194577779713</v>
       </c>
       <c r="F18">
-        <v>-0.231632987304371</v>
+        <v>-0.1498251439236995</v>
       </c>
       <c r="G18">
-        <v>8.239827565084084</v>
+        <v>9.770849329461811</v>
       </c>
       <c r="H18">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I18">
-        <v>-0.231632987304371</v>
+        <v>-0.1956315573526002</v>
       </c>
       <c r="J18">
-        <v>4186</v>
+        <v>3094</v>
       </c>
       <c r="K18">
-        <v>1066</v>
+        <v>988</v>
       </c>
       <c r="L18">
         <v>0</v>
@@ -1186,28 +1186,28 @@
         <v>5</v>
       </c>
       <c r="D19">
-        <v>8.239827565084084</v>
+        <v>8.158019721703413</v>
       </c>
       <c r="E19">
         <v>8.008194577779713</v>
       </c>
       <c r="F19">
-        <v>-0.231632987304371</v>
+        <v>-0.1498251439236995</v>
       </c>
       <c r="G19">
-        <v>8.239827565084084</v>
+        <v>9.770849329461811</v>
       </c>
       <c r="H19">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I19">
-        <v>-0.231632987304371</v>
+        <v>-0.1956315573526002</v>
       </c>
       <c r="J19">
-        <v>4186</v>
+        <v>3094</v>
       </c>
       <c r="K19">
-        <v>1066</v>
+        <v>988</v>
       </c>
       <c r="L19">
         <v>0</v>
@@ -1230,28 +1230,28 @@
         <v>3</v>
       </c>
       <c r="D20">
-        <v>8.246471719363614</v>
+        <v>8.164590474719805</v>
       </c>
       <c r="E20">
         <v>8.008194577779713</v>
       </c>
       <c r="F20">
-        <v>-0.2382771415839002</v>
+        <v>-0.1563958969400918</v>
       </c>
       <c r="G20">
-        <v>8.246471719363614</v>
+        <v>9.779428975120158</v>
       </c>
       <c r="H20">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I20">
-        <v>-0.2382771415839002</v>
+        <v>-0.2042112030109475</v>
       </c>
       <c r="J20">
-        <v>4576</v>
+        <v>3484</v>
       </c>
       <c r="K20">
-        <v>624</v>
+        <v>546</v>
       </c>
       <c r="L20">
         <v>52</v>
@@ -1274,28 +1274,28 @@
         <v>4</v>
       </c>
       <c r="D21">
-        <v>8.246471719363614</v>
+        <v>8.164590474719805</v>
       </c>
       <c r="E21">
         <v>8.008194577779713</v>
       </c>
       <c r="F21">
-        <v>-0.2382771415839002</v>
+        <v>-0.1563958969400918</v>
       </c>
       <c r="G21">
-        <v>8.246471719363614</v>
+        <v>9.779428975120158</v>
       </c>
       <c r="H21">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I21">
-        <v>-0.2382771415839002</v>
+        <v>-0.2042112030109475</v>
       </c>
       <c r="J21">
-        <v>4576</v>
+        <v>3484</v>
       </c>
       <c r="K21">
-        <v>624</v>
+        <v>546</v>
       </c>
       <c r="L21">
         <v>52</v>
@@ -1318,28 +1318,28 @@
         <v>5</v>
       </c>
       <c r="D22">
-        <v>8.246471719363614</v>
+        <v>8.164590474719805</v>
       </c>
       <c r="E22">
         <v>8.008194577779713</v>
       </c>
       <c r="F22">
-        <v>-0.2382771415839002</v>
+        <v>-0.1563958969400918</v>
       </c>
       <c r="G22">
-        <v>8.246471719363614</v>
+        <v>9.779428975120158</v>
       </c>
       <c r="H22">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I22">
-        <v>-0.2382771415839002</v>
+        <v>-0.2042112030109475</v>
       </c>
       <c r="J22">
-        <v>4576</v>
+        <v>3484</v>
       </c>
       <c r="K22">
-        <v>624</v>
+        <v>546</v>
       </c>
       <c r="L22">
         <v>52</v>
@@ -1362,28 +1362,28 @@
         <v>3</v>
       </c>
       <c r="D23">
-        <v>8.264423639186031</v>
+        <v>8.182499240644958</v>
       </c>
       <c r="E23">
         <v>8.008194577779713</v>
       </c>
       <c r="F23">
-        <v>-0.2562290614063176</v>
+        <v>-0.1743046628652447</v>
       </c>
       <c r="G23">
-        <v>8.264423639186031</v>
+        <v>9.802813032538349</v>
       </c>
       <c r="H23">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I23">
-        <v>-0.2562290614063176</v>
+        <v>-0.2275952604291387</v>
       </c>
       <c r="J23">
-        <v>4004</v>
+        <v>2912</v>
       </c>
       <c r="K23">
-        <v>1248</v>
+        <v>1170</v>
       </c>
       <c r="L23">
         <v>0</v>
@@ -1406,28 +1406,28 @@
         <v>3</v>
       </c>
       <c r="D24">
-        <v>8.264423639186031</v>
+        <v>8.182499240644958</v>
       </c>
       <c r="E24">
         <v>8.008194577779713</v>
       </c>
       <c r="F24">
-        <v>-0.2562290614063176</v>
+        <v>-0.1743046628652447</v>
       </c>
       <c r="G24">
-        <v>8.264423639186031</v>
+        <v>9.802813032538349</v>
       </c>
       <c r="H24">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I24">
-        <v>-0.2562290614063176</v>
+        <v>-0.2275952604291387</v>
       </c>
       <c r="J24">
-        <v>4004</v>
+        <v>2912</v>
       </c>
       <c r="K24">
-        <v>1248</v>
+        <v>1170</v>
       </c>
       <c r="L24">
         <v>0</v>
@@ -1450,28 +1450,28 @@
         <v>4</v>
       </c>
       <c r="D25">
-        <v>8.264423639186031</v>
+        <v>8.182499240644958</v>
       </c>
       <c r="E25">
         <v>8.008194577779713</v>
       </c>
       <c r="F25">
-        <v>-0.2562290614063176</v>
+        <v>-0.1743046628652447</v>
       </c>
       <c r="G25">
-        <v>8.264423639186031</v>
+        <v>9.802813032538349</v>
       </c>
       <c r="H25">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I25">
-        <v>-0.2562290614063176</v>
+        <v>-0.2275952604291387</v>
       </c>
       <c r="J25">
-        <v>4004</v>
+        <v>2912</v>
       </c>
       <c r="K25">
-        <v>1248</v>
+        <v>1170</v>
       </c>
       <c r="L25">
         <v>0</v>
@@ -1494,28 +1494,28 @@
         <v>4</v>
       </c>
       <c r="D26">
-        <v>8.264423639186031</v>
+        <v>8.182499240644958</v>
       </c>
       <c r="E26">
         <v>8.008194577779713</v>
       </c>
       <c r="F26">
-        <v>-0.2562290614063176</v>
+        <v>-0.1743046628652447</v>
       </c>
       <c r="G26">
-        <v>8.264423639186031</v>
+        <v>9.802813032538349</v>
       </c>
       <c r="H26">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I26">
-        <v>-0.2562290614063176</v>
+        <v>-0.2275952604291387</v>
       </c>
       <c r="J26">
-        <v>4004</v>
+        <v>2912</v>
       </c>
       <c r="K26">
-        <v>1248</v>
+        <v>1170</v>
       </c>
       <c r="L26">
         <v>0</v>
@@ -1538,28 +1538,28 @@
         <v>5</v>
       </c>
       <c r="D27">
-        <v>8.264423639186031</v>
+        <v>8.182499240644958</v>
       </c>
       <c r="E27">
         <v>8.008194577779713</v>
       </c>
       <c r="F27">
-        <v>-0.2562290614063176</v>
+        <v>-0.1743046628652447</v>
       </c>
       <c r="G27">
-        <v>8.264423639186031</v>
+        <v>9.802813032538349</v>
       </c>
       <c r="H27">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I27">
-        <v>-0.2562290614063176</v>
+        <v>-0.2275952604291387</v>
       </c>
       <c r="J27">
-        <v>4004</v>
+        <v>2912</v>
       </c>
       <c r="K27">
-        <v>1248</v>
+        <v>1170</v>
       </c>
       <c r="L27">
         <v>0</v>
@@ -1582,28 +1582,28 @@
         <v>5</v>
       </c>
       <c r="D28">
-        <v>8.264423639186031</v>
+        <v>8.182499240644958</v>
       </c>
       <c r="E28">
         <v>8.008194577779713</v>
       </c>
       <c r="F28">
-        <v>-0.2562290614063176</v>
+        <v>-0.1743046628652447</v>
       </c>
       <c r="G28">
-        <v>8.264423639186031</v>
+        <v>9.802813032538349</v>
       </c>
       <c r="H28">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I28">
-        <v>-0.2562290614063176</v>
+        <v>-0.2275952604291387</v>
       </c>
       <c r="J28">
-        <v>4004</v>
+        <v>2912</v>
       </c>
       <c r="K28">
-        <v>1248</v>
+        <v>1170</v>
       </c>
       <c r="L28">
         <v>0</v>
@@ -1626,28 +1626,28 @@
         <v>3</v>
       </c>
       <c r="D29">
-        <v>8.297393819166208</v>
+        <v>8.215585975785537</v>
       </c>
       <c r="E29">
         <v>8.008194577779713</v>
       </c>
       <c r="F29">
-        <v>-0.2891992413864948</v>
+        <v>-0.2073913980058233</v>
       </c>
       <c r="G29">
-        <v>8.297393819166208</v>
+        <v>9.846015457403437</v>
       </c>
       <c r="H29">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I29">
-        <v>-0.2891992413864948</v>
+        <v>-0.2707976852942267</v>
       </c>
       <c r="J29">
-        <v>4160</v>
+        <v>3068</v>
       </c>
       <c r="K29">
-        <v>1066</v>
+        <v>988</v>
       </c>
       <c r="L29">
         <v>26</v>
@@ -1670,28 +1670,28 @@
         <v>4</v>
       </c>
       <c r="D30">
-        <v>8.297393819166208</v>
+        <v>8.215585975785537</v>
       </c>
       <c r="E30">
         <v>8.008194577779713</v>
       </c>
       <c r="F30">
-        <v>-0.2891992413864948</v>
+        <v>-0.2073913980058233</v>
       </c>
       <c r="G30">
-        <v>8.297393819166208</v>
+        <v>9.846015457403437</v>
       </c>
       <c r="H30">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I30">
-        <v>-0.2891992413864948</v>
+        <v>-0.2707976852942267</v>
       </c>
       <c r="J30">
-        <v>4160</v>
+        <v>3068</v>
       </c>
       <c r="K30">
-        <v>1066</v>
+        <v>988</v>
       </c>
       <c r="L30">
         <v>26</v>
@@ -1714,28 +1714,28 @@
         <v>5</v>
       </c>
       <c r="D31">
-        <v>8.297393819166208</v>
+        <v>8.215585975785537</v>
       </c>
       <c r="E31">
         <v>8.008194577779713</v>
       </c>
       <c r="F31">
-        <v>-0.2891992413864948</v>
+        <v>-0.2073913980058233</v>
       </c>
       <c r="G31">
-        <v>8.297393819166208</v>
+        <v>9.846015457403437</v>
       </c>
       <c r="H31">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I31">
-        <v>-0.2891992413864948</v>
+        <v>-0.2707976852942267</v>
       </c>
       <c r="J31">
-        <v>4160</v>
+        <v>3068</v>
       </c>
       <c r="K31">
-        <v>1066</v>
+        <v>988</v>
       </c>
       <c r="L31">
         <v>26</v>
@@ -1758,28 +1758,28 @@
         <v>3</v>
       </c>
       <c r="D32">
-        <v>8.321989893268155</v>
+        <v>8.24006549472708</v>
       </c>
       <c r="E32">
         <v>8.008194577779713</v>
       </c>
       <c r="F32">
-        <v>-0.3137953154884414</v>
+        <v>-0.2318709169473667</v>
       </c>
       <c r="G32">
-        <v>8.321989893268155</v>
+        <v>9.877979160479976</v>
       </c>
       <c r="H32">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I32">
-        <v>-0.3137953154884414</v>
+        <v>-0.3027613883707652</v>
       </c>
       <c r="J32">
-        <v>3978</v>
+        <v>2886</v>
       </c>
       <c r="K32">
-        <v>1248</v>
+        <v>1170</v>
       </c>
       <c r="L32">
         <v>26</v>
@@ -1802,28 +1802,28 @@
         <v>4</v>
       </c>
       <c r="D33">
-        <v>8.321989893268155</v>
+        <v>8.24006549472708</v>
       </c>
       <c r="E33">
         <v>8.008194577779713</v>
       </c>
       <c r="F33">
-        <v>-0.3137953154884414</v>
+        <v>-0.2318709169473667</v>
       </c>
       <c r="G33">
-        <v>8.321989893268155</v>
+        <v>9.877979160479976</v>
       </c>
       <c r="H33">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I33">
-        <v>-0.3137953154884414</v>
+        <v>-0.3027613883707652</v>
       </c>
       <c r="J33">
-        <v>3978</v>
+        <v>2886</v>
       </c>
       <c r="K33">
-        <v>1248</v>
+        <v>1170</v>
       </c>
       <c r="L33">
         <v>26</v>
@@ -1846,28 +1846,28 @@
         <v>5</v>
       </c>
       <c r="D34">
-        <v>8.321989893268155</v>
+        <v>8.24006549472708</v>
       </c>
       <c r="E34">
         <v>8.008194577779713</v>
       </c>
       <c r="F34">
-        <v>-0.3137953154884414</v>
+        <v>-0.2318709169473667</v>
       </c>
       <c r="G34">
-        <v>8.321989893268155</v>
+        <v>9.877979160479976</v>
       </c>
       <c r="H34">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I34">
-        <v>-0.3137953154884414</v>
+        <v>-0.3027613883707652</v>
       </c>
       <c r="J34">
-        <v>3978</v>
+        <v>2886</v>
       </c>
       <c r="K34">
-        <v>1248</v>
+        <v>1170</v>
       </c>
       <c r="L34">
         <v>26</v>
@@ -1890,28 +1890,28 @@
         <v>3</v>
       </c>
       <c r="D35">
-        <v>8.332850745118947</v>
+        <v>8.250966107379142</v>
       </c>
       <c r="E35">
         <v>8.008194577779713</v>
       </c>
       <c r="F35">
-        <v>-0.3246561673392332</v>
+        <v>-0.2427715295994286</v>
       </c>
       <c r="G35">
-        <v>8.332850745118947</v>
+        <v>9.892212444516108</v>
       </c>
       <c r="H35">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I35">
-        <v>-0.3246561673392332</v>
+        <v>-0.3169946724068975</v>
       </c>
       <c r="J35">
-        <v>4446</v>
+        <v>3354</v>
       </c>
       <c r="K35">
-        <v>624</v>
+        <v>546</v>
       </c>
       <c r="L35">
         <v>182</v>
@@ -1934,28 +1934,28 @@
         <v>4</v>
       </c>
       <c r="D36">
-        <v>8.332850745118947</v>
+        <v>8.250966107379142</v>
       </c>
       <c r="E36">
         <v>8.008194577779713</v>
       </c>
       <c r="F36">
-        <v>-0.3246561673392332</v>
+        <v>-0.2427715295994286</v>
       </c>
       <c r="G36">
-        <v>8.332850745118947</v>
+        <v>9.892212444516108</v>
       </c>
       <c r="H36">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I36">
-        <v>-0.3246561673392332</v>
+        <v>-0.3169946724068975</v>
       </c>
       <c r="J36">
-        <v>4446</v>
+        <v>3354</v>
       </c>
       <c r="K36">
-        <v>624</v>
+        <v>546</v>
       </c>
       <c r="L36">
         <v>182</v>
@@ -1978,28 +1978,28 @@
         <v>5</v>
       </c>
       <c r="D37">
-        <v>8.332850745118947</v>
+        <v>8.250966107379142</v>
       </c>
       <c r="E37">
         <v>8.008194577779713</v>
       </c>
       <c r="F37">
-        <v>-0.3246561673392332</v>
+        <v>-0.2427715295994286</v>
       </c>
       <c r="G37">
-        <v>8.332850745118947</v>
+        <v>9.892212444516108</v>
       </c>
       <c r="H37">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="I37">
-        <v>-0.3246561673392332</v>
+        <v>-0.3169946724068975</v>
       </c>
       <c r="J37">
-        <v>4446</v>
+        <v>3354</v>
       </c>
       <c r="K37">
-        <v>624</v>
+        <v>546</v>
       </c>
       <c r="L37">
         <v>182</v>
@@ -2074,19 +2074,19 @@
         <v>3</v>
       </c>
       <c r="D2">
-        <v>8.187502353415857</v>
+        <v>9.721543496423253</v>
       </c>
       <c r="E2">
-        <v>8.008194577779713</v>
+        <v>9.575217772109211</v>
       </c>
       <c r="F2">
-        <v>-0.1793077756361434</v>
+        <v>-0.1463257243140426</v>
       </c>
       <c r="G2">
-        <v>3796</v>
+        <v>2704</v>
       </c>
       <c r="H2">
-        <v>1456</v>
+        <v>1378</v>
       </c>
     </row>
   </sheetData>

</xml_diff>